<commit_message>
ANS-006-168 - Mise en place des bonnes pratiques (SD, CS, VS) (#425)
* update CS 2.0.0

- suppression du cs
- Modification des titres et descriptions

* fix

* harmonisation CS/VS

* maj CS/VS

* update vs

* harmonisation extensions/instances

* update description 68d1bf833b993e1dae40ddda88339134f17ccd58
</commit_message>
<xml_diff>
--- a/main/ig/CodeSystem-tddui-identifier.xlsx
+++ b/main/ig/CodeSystem-tddui-identifier.xlsx
@@ -42,7 +42,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>TDDUI FR Core CodeSystem v2-0203</t>
+    <t>TDDUI Patient Identifier</t>
   </si>
   <si>
     <t>Status</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-05T14:50:20+00:00</t>
+    <t>2026-02-05T15:15:02+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -84,7 +84,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>TDDUI Patient's identifier</t>
+    <t>CodeSystem pour la définition des codes d'identifiant de l'usager</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>